<commit_message>
chore: pick migration to correct ledgers + MASTER.md update, 654 tests pass
</commit_message>
<xml_diff>
--- a/data/gated_research/lol.xlsx
+++ b/data/gated_research/lol.xlsx
@@ -300,8 +300,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ11" headerRowCount="1">
-  <autoFilter ref="A1:CQ11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PicksLedger" displayName="PicksLedger" ref="A1:CQ7" headerRowCount="1">
+  <autoFilter ref="A1:CQ7"/>
   <tableColumns count="95">
     <tableColumn id="1" name="pick_id"/>
     <tableColumn id="2" name="created_at_utc"/>
@@ -754,19 +754,19 @@
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6">
-        <f>COUNTA('Picks'!$A$2:$A$11)</f>
+        <f>COUNTA('Picks'!$A$2:$A$7)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$11,"open")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$7,"open")</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Picks'!$U$2:$U$11,"settled")</f>
+        <f>COUNTIF('Picks'!$U$2:$U$7,"settled")</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>IF(COUNTIFS('Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"win")+COUNTIFS('Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
+        <f>IF(COUNTIFS('Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"win")+COUNTIFS('Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"loss")&gt;=$L$2,"Ready","Insufficient sample")</f>
         <v/>
       </c>
     </row>
@@ -794,19 +794,19 @@
     </row>
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6">
-        <f>COUNTIF('Picks'!$BX$2:$BX$11,"&gt;0")</f>
+        <f>COUNTIF('Picks'!$BX$2:$BX$7,"&gt;0")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Picks'!$BX$2:$BX$11,"&gt;0",'Picks'!$V$2:$V$11,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$11,"&gt;0",'Picks'!$V$2:$V$11,"loss")</f>
+        <f>COUNTIFS('Picks'!$BX$2:$BX$7,"&gt;0",'Picks'!$V$2:$V$7,"win")&amp;"-"&amp;COUNTIFS('Picks'!$BX$2:$BX$7,"&gt;0",'Picks'!$V$2:$V$7,"loss")</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$11,"&gt;0",'Picks'!$V$2:$V$11,"win")/(COUNTIFS('Picks'!$BX$2:$BX$11,"&gt;0",'Picks'!$V$2:$V$11,"win")+COUNTIFS('Picks'!$BX$2:$BX$11,"&gt;0",'Picks'!$V$2:$V$11,"loss")),0)</f>
+        <f>IFERROR(COUNTIFS('Picks'!$BX$2:$BX$7,"&gt;0",'Picks'!$V$2:$V$7,"win")/(COUNTIFS('Picks'!$BX$2:$BX$7,"&gt;0",'Picks'!$V$2:$V$7,"win")+COUNTIFS('Picks'!$BX$2:$BX$7,"&gt;0",'Picks'!$V$2:$V$7,"loss")),0)</f>
         <v/>
       </c>
       <c r="G7" s="7">
-        <f>IFERROR(SUM('Picks'!$BY$2:$BY$11)/SUM('Picks'!$BX$2:$BX$11),0)</f>
+        <f>IFERROR(SUM('Picks'!$BY$2:$BY$7)/SUM('Picks'!$BX$2:$BX$7),0)</f>
         <v/>
       </c>
     </row>
@@ -834,19 +834,19 @@
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="8">
-        <f>SUM('Picks'!$BY$2:$BY$11)</f>
+        <f>SUM('Picks'!$BY$2:$BY$7)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$11,"&lt;&gt;",'Picks'!$AB$2:$AB$11),0)</f>
+        <f>IFERROR(AVERAGEIF('Picks'!$AB$2:$AB$7,"&lt;&gt;",'Picks'!$AB$2:$AB$7),0)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>COUNTIFS('Picks'!$AM$2:$AM$11,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$11,"settled")</f>
+        <f>COUNTIFS('Picks'!$AM$2:$AM$7,"QUALIFIED_SHADOW_CALL",'Picks'!$U$2:$U$7,"settled")</f>
         <v/>
       </c>
       <c r="G10" s="8">
-        <f>SUMIFS('Picks'!$AC$2:$AC$11,'Picks'!$AM$2:$AM$11,"QUALIFIED_SHADOW_CALL")</f>
+        <f>SUMIFS('Picks'!$AC$2:$AC$7,'Picks'!$AM$2:$AM$7,"QUALIFIED_SHADOW_CALL")</f>
         <v/>
       </c>
     </row>
@@ -901,15 +901,15 @@
         </is>
       </c>
       <c r="B14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A14,'Picks'!$U$2:$U$11,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A14,'Picks'!$U$2:$U$7,"settled")</f>
         <v/>
       </c>
       <c r="C14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A14,'Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A14,'Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"win")</f>
         <v/>
       </c>
       <c r="D14" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A14,'Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A14,'Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"loss")</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -917,11 +917,11 @@
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$11,'Picks'!$H$2:$H$11,$A14)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$7,'Picks'!$H$2:$H$7,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$11,'Picks'!$H$2:$H$11,$A14,'Picks'!$U$2:$U$11,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$7,'Picks'!$H$2:$H$7,$A14,'Picks'!$U$2:$U$7,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -932,15 +932,15 @@
         </is>
       </c>
       <c r="B15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A15,'Picks'!$U$2:$U$11,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A15,'Picks'!$U$2:$U$7,"settled")</f>
         <v/>
       </c>
       <c r="C15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A15,'Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A15,'Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"win")</f>
         <v/>
       </c>
       <c r="D15" s="18">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A15,'Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A15,'Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"loss")</f>
         <v/>
       </c>
       <c r="E15" s="19">
@@ -948,11 +948,11 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>SUMIFS('Picks'!$BY$2:$BY$11,'Picks'!$H$2:$H$11,$A15)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$7,'Picks'!$H$2:$H$7,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$11,'Picks'!$H$2:$H$11,$A15,'Picks'!$U$2:$U$11,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$7,'Picks'!$H$2:$H$7,$A15,'Picks'!$U$2:$U$7,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -963,15 +963,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A16,'Picks'!$U$2:$U$11,"settled")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A16,'Picks'!$U$2:$U$7,"settled")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A16,'Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"win")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A16,'Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"win")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIFS('Picks'!$H$2:$H$11,$A16,'Picks'!$U$2:$U$11,"settled",'Picks'!$V$2:$V$11,"loss")</f>
+        <f>COUNTIFS('Picks'!$H$2:$H$7,$A16,'Picks'!$U$2:$U$7,"settled",'Picks'!$V$2:$V$7,"loss")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -979,11 +979,11 @@
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>SUMIFS('Picks'!$BY$2:$BY$11,'Picks'!$H$2:$H$11,$A16)</f>
+        <f>SUMIFS('Picks'!$BY$2:$BY$7,'Picks'!$H$2:$H$7,$A16)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$11,'Picks'!$H$2:$H$11,$A16,'Picks'!$U$2:$U$11,"settled"),0)</f>
+        <f>IFERROR(AVERAGEIFS('Picks'!$AB$2:$AB$7,'Picks'!$H$2:$H$7,$A16,'Picks'!$U$2:$U$7,"settled"),0)</f>
         <v/>
       </c>
     </row>
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CQ11"/>
+  <dimension ref="A1:CQ7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3291,1074 +3291,6 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="24" t="inlineStr">
-        <is>
-          <t>3e4847e84b4f42a7</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:11.967172Z</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T10:00:00Z</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>67511</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="inlineStr">
-        <is>
-          <t>LOL</t>
-        </is>
-      </c>
-      <c r="F8" s="24" t="inlineStr">
-        <is>
-          <t>Dplus KIA Challengers</t>
-        </is>
-      </c>
-      <c r="G8" s="24" t="inlineStr">
-        <is>
-          <t>DN SOOPers Challengers</t>
-        </is>
-      </c>
-      <c r="H8" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I8" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J8" s="25" t="n"/>
-      <c r="K8" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L8" s="26" t="n">
-        <v>-223</v>
-      </c>
-      <c r="M8" s="27" t="n">
-        <v>1.44843</v>
-      </c>
-      <c r="N8" s="28" t="n">
-        <v>0.690402</v>
-      </c>
-      <c r="O8" s="28" t="n">
-        <v>0.703159</v>
-      </c>
-      <c r="P8" s="28" t="n"/>
-      <c r="Q8" s="28" t="n">
-        <v>0.012757</v>
-      </c>
-      <c r="R8" s="26" t="n">
-        <v>26</v>
-      </c>
-      <c r="S8" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="T8" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U8" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V8" s="24" t="n"/>
-      <c r="W8" s="26" t="n"/>
-      <c r="X8" s="26" t="n"/>
-      <c r="Y8" s="25" t="n"/>
-      <c r="Z8" s="26" t="n"/>
-      <c r="AA8" s="28" t="n"/>
-      <c r="AB8" s="28" t="n"/>
-      <c r="AC8" s="30" t="n"/>
-      <c r="AD8" s="24" t="n"/>
-      <c r="AE8" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.6900 (market_slug=aec-lol-dnsc-dkc-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF8" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG8" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH8" s="24" t="n"/>
-      <c r="AI8" s="31" t="n"/>
-      <c r="AJ8" s="31" t="n"/>
-      <c r="AK8" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL8" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM8" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN8" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO8" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP8" s="24" t="inlineStr">
-        <is>
-          <t>Dplus KIA Challengers</t>
-        </is>
-      </c>
-      <c r="AQ8" s="24" t="inlineStr">
-        <is>
-          <t>Dplus KIA Challengers</t>
-        </is>
-      </c>
-      <c r="AR8" s="24" t="inlineStr">
-        <is>
-          <t>Dplus KIA Challengers</t>
-        </is>
-      </c>
-      <c r="AS8" s="24" t="inlineStr">
-        <is>
-          <t>DN SOOPers Challengers</t>
-        </is>
-      </c>
-      <c r="AT8" s="24" t="inlineStr">
-        <is>
-          <t>DN SOOPers Challengers</t>
-        </is>
-      </c>
-      <c r="AU8" s="24" t="inlineStr">
-        <is>
-          <t>DN SOOPers Challengers</t>
-        </is>
-      </c>
-      <c r="AV8" s="24" t="n"/>
-      <c r="AW8" s="24" t="n"/>
-      <c r="AX8" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY8" s="24" t="n"/>
-      <c r="AZ8" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA8" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BB8" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC8" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD8" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BE8" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF8" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG8" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH8" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:05.228074Z</t>
-        </is>
-      </c>
-      <c r="BI8" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ8" s="25" t="n"/>
-      <c r="BK8" s="26" t="n">
-        <v>-223</v>
-      </c>
-      <c r="BL8" s="27" t="n">
-        <v>1.44843</v>
-      </c>
-      <c r="BM8" s="28" t="n">
-        <v>0.690402</v>
-      </c>
-      <c r="BN8" s="28" t="n"/>
-      <c r="BO8" s="28" t="n"/>
-      <c r="BP8" s="25" t="n"/>
-      <c r="BQ8" s="27" t="n"/>
-      <c r="BR8" s="28" t="n"/>
-      <c r="BS8" s="28" t="n"/>
-      <c r="BT8" s="28" t="n"/>
-      <c r="BU8" s="25" t="n"/>
-      <c r="BV8" s="29" t="n"/>
-      <c r="BW8" s="24" t="n"/>
-      <c r="BX8" s="30" t="n"/>
-      <c r="BY8" s="27" t="n"/>
-      <c r="BZ8" s="24" t="n"/>
-      <c r="CA8" s="31" t="n"/>
-      <c r="CB8" s="24" t="n"/>
-      <c r="CC8" s="24" t="n"/>
-      <c r="CD8" s="24" t="n"/>
-      <c r="CE8" s="24" t="n"/>
-      <c r="CF8" s="24" t="n"/>
-      <c r="CG8" s="24" t="n"/>
-      <c r="CH8" s="24" t="n"/>
-      <c r="CI8" s="24" t="n"/>
-      <c r="CJ8" s="24" t="n"/>
-      <c r="CK8" s="24" t="n"/>
-      <c r="CL8" s="24" t="n"/>
-      <c r="CM8" s="24" t="n"/>
-      <c r="CN8" s="24" t="n"/>
-      <c r="CO8" s="24" t="n"/>
-      <c r="CP8" s="24" t="n"/>
-      <c r="CQ8" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="24" t="inlineStr">
-        <is>
-          <t>fae1fd8b12114e02</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:11.967172Z</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T10:30:00Z</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>67515</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="inlineStr">
-        <is>
-          <t>LOL</t>
-        </is>
-      </c>
-      <c r="F9" s="24" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>Nongshim Red Force</t>
-        </is>
-      </c>
-      <c r="H9" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I9" s="24" t="inlineStr">
-        <is>
-          <t>away</t>
-        </is>
-      </c>
-      <c r="J9" s="25" t="n"/>
-      <c r="K9" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L9" s="26" t="n">
-        <v>-163</v>
-      </c>
-      <c r="M9" s="27" t="n">
-        <v>1.613497</v>
-      </c>
-      <c r="N9" s="28" t="n">
-        <v>0.619772</v>
-      </c>
-      <c r="O9" s="28" t="n">
-        <v>0.746312</v>
-      </c>
-      <c r="P9" s="28" t="n"/>
-      <c r="Q9" s="28" t="n">
-        <v>0.12654</v>
-      </c>
-      <c r="R9" s="26" t="n">
-        <v>83</v>
-      </c>
-      <c r="S9" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="T9" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U9" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V9" s="24" t="n"/>
-      <c r="W9" s="26" t="n"/>
-      <c r="X9" s="26" t="n"/>
-      <c r="Y9" s="25" t="n"/>
-      <c r="Z9" s="26" t="n"/>
-      <c r="AA9" s="28" t="n"/>
-      <c r="AB9" s="28" t="n"/>
-      <c r="AC9" s="30" t="n"/>
-      <c r="AD9" s="24" t="n"/>
-      <c r="AE9" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.6200 (market_slug=aec-lol-ns-t1-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF9" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG9" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH9" s="24" t="n"/>
-      <c r="AI9" s="31" t="n"/>
-      <c r="AJ9" s="31" t="n"/>
-      <c r="AK9" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL9" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM9" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN9" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO9" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP9" s="24" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="AQ9" s="24" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="AR9" s="24" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="AS9" s="24" t="inlineStr">
-        <is>
-          <t>Nongshim Red Force</t>
-        </is>
-      </c>
-      <c r="AT9" s="24" t="inlineStr">
-        <is>
-          <t>Nongshim Red Force</t>
-        </is>
-      </c>
-      <c r="AU9" s="24" t="inlineStr">
-        <is>
-          <t>Nongshim Red Force</t>
-        </is>
-      </c>
-      <c r="AV9" s="24" t="n"/>
-      <c r="AW9" s="24" t="n"/>
-      <c r="AX9" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY9" s="24" t="n"/>
-      <c r="AZ9" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA9" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BB9" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC9" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD9" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BE9" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF9" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG9" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH9" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:05.711202Z</t>
-        </is>
-      </c>
-      <c r="BI9" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ9" s="25" t="n"/>
-      <c r="BK9" s="26" t="n">
-        <v>-163</v>
-      </c>
-      <c r="BL9" s="27" t="n">
-        <v>1.613497</v>
-      </c>
-      <c r="BM9" s="28" t="n">
-        <v>0.619772</v>
-      </c>
-      <c r="BN9" s="28" t="n"/>
-      <c r="BO9" s="28" t="n"/>
-      <c r="BP9" s="25" t="n"/>
-      <c r="BQ9" s="27" t="n"/>
-      <c r="BR9" s="28" t="n"/>
-      <c r="BS9" s="28" t="n"/>
-      <c r="BT9" s="28" t="n"/>
-      <c r="BU9" s="25" t="n"/>
-      <c r="BV9" s="29" t="n"/>
-      <c r="BW9" s="24" t="n"/>
-      <c r="BX9" s="30" t="n"/>
-      <c r="BY9" s="27" t="n"/>
-      <c r="BZ9" s="24" t="n"/>
-      <c r="CA9" s="31" t="n"/>
-      <c r="CB9" s="24" t="n"/>
-      <c r="CC9" s="24" t="n"/>
-      <c r="CD9" s="24" t="n"/>
-      <c r="CE9" s="24" t="n"/>
-      <c r="CF9" s="24" t="n"/>
-      <c r="CG9" s="24" t="n"/>
-      <c r="CH9" s="24" t="n"/>
-      <c r="CI9" s="24" t="n"/>
-      <c r="CJ9" s="24" t="n"/>
-      <c r="CK9" s="24" t="n"/>
-      <c r="CL9" s="24" t="n"/>
-      <c r="CM9" s="24" t="n"/>
-      <c r="CN9" s="24" t="n"/>
-      <c r="CO9" s="24" t="n"/>
-      <c r="CP9" s="24" t="n"/>
-      <c r="CQ9" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="24" t="inlineStr">
-        <is>
-          <t>931a342a52074e57</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:11.967172Z</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T15:00:00Z</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
-          <t>67566</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>LOL</t>
-        </is>
-      </c>
-      <c r="F10" s="24" t="inlineStr">
-        <is>
-          <t>Shifters</t>
-        </is>
-      </c>
-      <c r="G10" s="24" t="inlineStr">
-        <is>
-          <t>Natus Vincere</t>
-        </is>
-      </c>
-      <c r="H10" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I10" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J10" s="25" t="n"/>
-      <c r="K10" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L10" s="26" t="n">
-        <v>-233</v>
-      </c>
-      <c r="M10" s="27" t="n">
-        <v>1.429185</v>
-      </c>
-      <c r="N10" s="28" t="n">
-        <v>0.6997</v>
-      </c>
-      <c r="O10" s="28" t="n">
-        <v>0.74664</v>
-      </c>
-      <c r="P10" s="28" t="n"/>
-      <c r="Q10" s="28" t="n">
-        <v>0.04694</v>
-      </c>
-      <c r="R10" s="26" t="n">
-        <v>43</v>
-      </c>
-      <c r="S10" s="29" t="n">
-        <v>2</v>
-      </c>
-      <c r="T10" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U10" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V10" s="24" t="n"/>
-      <c r="W10" s="26" t="n"/>
-      <c r="X10" s="26" t="n"/>
-      <c r="Y10" s="25" t="n"/>
-      <c r="Z10" s="26" t="n"/>
-      <c r="AA10" s="28" t="n"/>
-      <c r="AB10" s="28" t="n"/>
-      <c r="AC10" s="30" t="n"/>
-      <c r="AD10" s="24" t="n"/>
-      <c r="AE10" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.7000 (market_slug=aec-lol-navi-shft-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF10" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG10" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH10" s="24" t="n"/>
-      <c r="AI10" s="31" t="n"/>
-      <c r="AJ10" s="31" t="n"/>
-      <c r="AK10" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL10" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM10" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN10" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO10" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP10" s="24" t="inlineStr">
-        <is>
-          <t>Shifters</t>
-        </is>
-      </c>
-      <c r="AQ10" s="24" t="inlineStr">
-        <is>
-          <t>Shifters</t>
-        </is>
-      </c>
-      <c r="AR10" s="24" t="inlineStr">
-        <is>
-          <t>Shifters</t>
-        </is>
-      </c>
-      <c r="AS10" s="24" t="inlineStr">
-        <is>
-          <t>Natus Vincere</t>
-        </is>
-      </c>
-      <c r="AT10" s="24" t="inlineStr">
-        <is>
-          <t>Natus Vincere</t>
-        </is>
-      </c>
-      <c r="AU10" s="24" t="inlineStr">
-        <is>
-          <t>Natus Vincere</t>
-        </is>
-      </c>
-      <c r="AV10" s="24" t="n"/>
-      <c r="AW10" s="24" t="n"/>
-      <c r="AX10" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY10" s="24" t="n"/>
-      <c r="AZ10" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA10" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BB10" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC10" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD10" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BE10" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF10" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG10" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH10" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:06.165699Z</t>
-        </is>
-      </c>
-      <c r="BI10" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ10" s="25" t="n"/>
-      <c r="BK10" s="26" t="n">
-        <v>-233</v>
-      </c>
-      <c r="BL10" s="27" t="n">
-        <v>1.429185</v>
-      </c>
-      <c r="BM10" s="28" t="n">
-        <v>0.6997</v>
-      </c>
-      <c r="BN10" s="28" t="n"/>
-      <c r="BO10" s="28" t="n"/>
-      <c r="BP10" s="25" t="n"/>
-      <c r="BQ10" s="27" t="n"/>
-      <c r="BR10" s="28" t="n"/>
-      <c r="BS10" s="28" t="n"/>
-      <c r="BT10" s="28" t="n"/>
-      <c r="BU10" s="25" t="n"/>
-      <c r="BV10" s="29" t="n"/>
-      <c r="BW10" s="24" t="n"/>
-      <c r="BX10" s="30" t="n"/>
-      <c r="BY10" s="27" t="n"/>
-      <c r="BZ10" s="24" t="n"/>
-      <c r="CA10" s="31" t="n"/>
-      <c r="CB10" s="24" t="n"/>
-      <c r="CC10" s="24" t="n"/>
-      <c r="CD10" s="24" t="n"/>
-      <c r="CE10" s="24" t="n"/>
-      <c r="CF10" s="24" t="n"/>
-      <c r="CG10" s="24" t="n"/>
-      <c r="CH10" s="24" t="n"/>
-      <c r="CI10" s="24" t="n"/>
-      <c r="CJ10" s="24" t="n"/>
-      <c r="CK10" s="24" t="n"/>
-      <c r="CL10" s="24" t="n"/>
-      <c r="CM10" s="24" t="n"/>
-      <c r="CN10" s="24" t="n"/>
-      <c r="CO10" s="24" t="n"/>
-      <c r="CP10" s="24" t="n"/>
-      <c r="CQ10" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
-        <is>
-          <t>139023a3e3174887</t>
-        </is>
-      </c>
-      <c r="B11" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:11.967172Z</t>
-        </is>
-      </c>
-      <c r="C11" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-03T20:00:00Z</t>
-        </is>
-      </c>
-      <c r="D11" s="24" t="inlineStr">
-        <is>
-          <t>67937</t>
-        </is>
-      </c>
-      <c r="E11" s="24" t="inlineStr">
-        <is>
-          <t>LOL</t>
-        </is>
-      </c>
-      <c r="F11" s="24" t="inlineStr">
-        <is>
-          <t>Docta Esports</t>
-        </is>
-      </c>
-      <c r="G11" s="24" t="inlineStr">
-        <is>
-          <t>Volticons</t>
-        </is>
-      </c>
-      <c r="H11" s="24" t="inlineStr">
-        <is>
-          <t>moneyline</t>
-        </is>
-      </c>
-      <c r="I11" s="24" t="inlineStr">
-        <is>
-          <t>home</t>
-        </is>
-      </c>
-      <c r="J11" s="25" t="n"/>
-      <c r="K11" s="24" t="inlineStr">
-        <is>
-          <t>polymarket_us</t>
-        </is>
-      </c>
-      <c r="L11" s="26" t="n">
-        <v>-144</v>
-      </c>
-      <c r="M11" s="27" t="n">
-        <v>1.694444</v>
-      </c>
-      <c r="N11" s="28" t="n">
-        <v>0.590164</v>
-      </c>
-      <c r="O11" s="28" t="n">
-        <v>0.649674</v>
-      </c>
-      <c r="P11" s="28" t="n"/>
-      <c r="Q11" s="28" t="n">
-        <v>0.05951</v>
-      </c>
-      <c r="R11" s="26" t="n">
-        <v>50</v>
-      </c>
-      <c r="S11" s="29" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="T11" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="U11" s="24" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="V11" s="24" t="n"/>
-      <c r="W11" s="26" t="n"/>
-      <c r="X11" s="26" t="n"/>
-      <c r="Y11" s="25" t="n"/>
-      <c r="Z11" s="26" t="n"/>
-      <c r="AA11" s="28" t="n"/>
-      <c r="AB11" s="28" t="n"/>
-      <c r="AC11" s="30" t="n"/>
-      <c r="AD11" s="24" t="n"/>
-      <c r="AE11" s="31" t="inlineStr">
-        <is>
-          <t>Neutral Elo baseline; executable ask 0.5900 (market_slug=aec-lol-vtc-doh-2026-08-03).</t>
-        </is>
-      </c>
-      <c r="AF11" s="31" t="inlineStr">
-        <is>
-          <t>Config-promoted esports baseline; gates enforced at log time.</t>
-        </is>
-      </c>
-      <c r="AG11" s="24" t="inlineStr">
-        <is>
-          <t>not_applicable</t>
-        </is>
-      </c>
-      <c r="AH11" s="24" t="n"/>
-      <c r="AI11" s="31" t="n"/>
-      <c r="AJ11" s="31" t="n"/>
-      <c r="AK11" s="24" t="inlineStr">
-        <is>
-          <t>model_qualified</t>
-        </is>
-      </c>
-      <c r="AL11" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AM11" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED_SHADOW_CALL</t>
-        </is>
-      </c>
-      <c r="AN11" s="24" t="inlineStr">
-        <is>
-          <t>CALL</t>
-        </is>
-      </c>
-      <c r="AO11" s="24" t="inlineStr">
-        <is>
-          <t>QUALIFIED</t>
-        </is>
-      </c>
-      <c r="AP11" s="24" t="inlineStr">
-        <is>
-          <t>Docta Esports</t>
-        </is>
-      </c>
-      <c r="AQ11" s="24" t="inlineStr">
-        <is>
-          <t>Docta Esports</t>
-        </is>
-      </c>
-      <c r="AR11" s="24" t="inlineStr">
-        <is>
-          <t>Docta Esports</t>
-        </is>
-      </c>
-      <c r="AS11" s="24" t="inlineStr">
-        <is>
-          <t>Volticons</t>
-        </is>
-      </c>
-      <c r="AT11" s="24" t="inlineStr">
-        <is>
-          <t>Volticons</t>
-        </is>
-      </c>
-      <c r="AU11" s="24" t="inlineStr">
-        <is>
-          <t>Volticons</t>
-        </is>
-      </c>
-      <c r="AV11" s="24" t="n"/>
-      <c r="AW11" s="24" t="n"/>
-      <c r="AX11" s="24" t="inlineStr">
-        <is>
-          <t>statistical_model</t>
-        </is>
-      </c>
-      <c r="AY11" s="24" t="n"/>
-      <c r="AZ11" s="24" t="inlineStr">
-        <is>
-          <t>shadow_qualified</t>
-        </is>
-      </c>
-      <c r="BA11" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BB11" s="24" t="inlineStr">
-        <is>
-          <t>neutral_elo</t>
-        </is>
-      </c>
-      <c r="BC11" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BD11" s="24" t="inlineStr">
-        <is>
-          <t>7a524d830547b62f7f9c941aadbdf0fc52dbd67b16b701b974612cc0a7507dd8</t>
-        </is>
-      </c>
-      <c r="BE11" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BF11" s="24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="BG11" s="24" t="inlineStr">
-        <is>
-          <t>lol-tiered-elo-v5</t>
-        </is>
-      </c>
-      <c r="BH11" s="24" t="inlineStr">
-        <is>
-          <t>2026-08-02T16:53:09.518110Z</t>
-        </is>
-      </c>
-      <c r="BI11" s="24" t="inlineStr">
-        <is>
-          <t>["same_event","same_team_same_day","same_league_same_day"]</t>
-        </is>
-      </c>
-      <c r="BJ11" s="25" t="n"/>
-      <c r="BK11" s="26" t="n">
-        <v>-144</v>
-      </c>
-      <c r="BL11" s="27" t="n">
-        <v>1.694444</v>
-      </c>
-      <c r="BM11" s="28" t="n">
-        <v>0.590164</v>
-      </c>
-      <c r="BN11" s="28" t="n"/>
-      <c r="BO11" s="28" t="n"/>
-      <c r="BP11" s="25" t="n"/>
-      <c r="BQ11" s="27" t="n"/>
-      <c r="BR11" s="28" t="n"/>
-      <c r="BS11" s="28" t="n"/>
-      <c r="BT11" s="28" t="n"/>
-      <c r="BU11" s="25" t="n"/>
-      <c r="BV11" s="29" t="n"/>
-      <c r="BW11" s="24" t="n"/>
-      <c r="BX11" s="30" t="n"/>
-      <c r="BY11" s="27" t="n"/>
-      <c r="BZ11" s="24" t="n"/>
-      <c r="CA11" s="31" t="n"/>
-      <c r="CB11" s="24" t="n"/>
-      <c r="CC11" s="24" t="n"/>
-      <c r="CD11" s="24" t="n"/>
-      <c r="CE11" s="24" t="n"/>
-      <c r="CF11" s="24" t="n"/>
-      <c r="CG11" s="24" t="n"/>
-      <c r="CH11" s="24" t="n"/>
-      <c r="CI11" s="24" t="n"/>
-      <c r="CJ11" s="24" t="n"/>
-      <c r="CK11" s="24" t="n"/>
-      <c r="CL11" s="24" t="n"/>
-      <c r="CM11" s="24" t="n"/>
-      <c r="CN11" s="24" t="n"/>
-      <c r="CO11" s="24" t="n"/>
-      <c r="CP11" s="24" t="n"/>
-      <c r="CQ11" s="24" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>